<commit_message>
added time tracking to excel
</commit_message>
<xml_diff>
--- a/data/generated_schedule.xlsx
+++ b/data/generated_schedule.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,10 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
   <fills count="20">
     <fill>
@@ -47,8 +51,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008497B0"/>
-        <bgColor rgb="008497B0"/>
+        <fgColor rgb="00A9D18E"/>
+        <bgColor rgb="00A9D18E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF9000"/>
+        <bgColor rgb="00BF9000"/>
       </patternFill>
     </fill>
     <fill>
@@ -59,8 +69,56 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BF9000"/>
-        <bgColor rgb="00BF9000"/>
+        <fgColor rgb="009E480E"/>
+        <bgColor rgb="009E480E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+        <bgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008497B0"/>
+        <bgColor rgb="008497B0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A64D79"/>
+        <bgColor rgb="00A64D79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00674EA7"/>
+        <bgColor rgb="00674EA7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C00"/>
+        <bgColor rgb="00833C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6B656"/>
+        <bgColor rgb="00D6B656"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+        <bgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6699"/>
+        <bgColor rgb="00FF6699"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,26 +129,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
-        <bgColor rgb="002E75B6"/>
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A9D18E"/>
-        <bgColor rgb="00A9D18E"/>
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00833C00"/>
-        <bgColor rgb="00833C00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00375623"/>
-        <bgColor rgb="00375623"/>
+        <fgColor rgb="00ED7D31"/>
+        <bgColor rgb="00ED7D31"/>
       </patternFill>
     </fill>
     <fill>
@@ -101,56 +153,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="009E480E"/>
-        <bgColor rgb="009E480E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
-        <bgColor rgb="00ED7D31"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00548235"/>
-        <bgColor rgb="00548235"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00674EA7"/>
-        <bgColor rgb="00674EA7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A64D79"/>
-        <bgColor rgb="00A64D79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6B656"/>
-        <bgColor rgb="00D6B656"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF6699"/>
-        <bgColor rgb="00FF6699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
-        <bgColor rgb="00C00000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -166,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -180,54 +184,73 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -593,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -738,122 +761,122 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Charlie
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Grace
-(7:30-9:15 AM)</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
           <t>Drew
 (7:30-12:00 PM)</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Ivanna
+(7:30-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Laila
+(7:30-11:00 AM)</t>
+        </is>
+      </c>
       <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Olivia R
+(7:30-10:30 AM)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Grace
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Naisha
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Ratna
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>Arya
+(7:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Olivia R
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>Caroline G
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>Mia
+(7:30-10:30 AM)</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Ratna
 (7:30-11:00 AM)</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Ivanna
+      <c r="N3" s="13" t="inlineStr">
+        <is>
+          <t>Keira
+(7:30-9:00 AM)</t>
+        </is>
+      </c>
+      <c r="O3" s="14" t="inlineStr">
+        <is>
+          <t>Reese
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Laila
 (7:30-12:30 PM)</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="Q3" s="15" t="inlineStr">
+        <is>
+          <t>Alex
+(7:30-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="R3" s="16" t="inlineStr">
         <is>
           <t>Caroline S
 (7:30-11:00 AM)</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(7:30-9:00 AM)</t>
-        </is>
-      </c>
-      <c r="I3" s="10" t="inlineStr">
-        <is>
-          <t>Laila
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="inlineStr">
-        <is>
-          <t>Olivia D
-(7:30-9:15 AM)</t>
-        </is>
-      </c>
-      <c r="K3" s="12" t="inlineStr">
-        <is>
-          <t>Naisha
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="L3" s="13" t="inlineStr">
-        <is>
-          <t>Olivia R
-(7:30-10:45 AM)</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>Ratna
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Arya
 (7:30-11:00 AM)</t>
         </is>
       </c>
-      <c r="N3" s="14" t="inlineStr">
-        <is>
-          <t>Arya
-(7:30-10:30 AM)</t>
-        </is>
-      </c>
-      <c r="O3" s="10" t="inlineStr">
-        <is>
-          <t>Laila
-(7:30-1:00 PM)</t>
-        </is>
-      </c>
-      <c r="P3" s="15" t="inlineStr">
-        <is>
-          <t>Mia
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="Q3" s="16" t="inlineStr">
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>Caroline G
 (7:30-9:30 AM)</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
-        <is>
-          <t>Ratna
-(7:30-9:00 AM)</t>
-        </is>
-      </c>
-      <c r="S3" s="17" t="inlineStr">
-        <is>
-          <t>Alex
-(7:30-11:15 AM)</t>
-        </is>
-      </c>
-      <c r="T3" s="18" t="inlineStr">
-        <is>
-          <t>Reese
-(7:30-9:00 AM)</t>
-        </is>
-      </c>
-      <c r="U3" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(7:30-9:30 AM)</t>
+      <c r="U3" s="17" t="inlineStr">
+        <is>
+          <t>Charlie
+(7:30-10:00 AM)</t>
         </is>
       </c>
     </row>
@@ -870,36 +893,36 @@
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="V5" s="19" t="inlineStr">
+      <c r="V5" s="16" t="inlineStr">
+        <is>
+          <t>Caroline S
+(8:00-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="W5" s="12" t="inlineStr">
+        <is>
+          <t>Mia
+(8:00-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="X5" s="17" t="inlineStr">
+        <is>
+          <t>Charlie
+(8:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="Y5" s="18" t="inlineStr">
+        <is>
+          <t>Olivia D
+(8:00-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="Z5" s="19" t="inlineStr">
         <is>
           <t>Abby
 (8:00-12:30 PM)</t>
         </is>
       </c>
-      <c r="W5" s="3" t="inlineStr">
-        <is>
-          <t>Charlie
-(8:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="X5" s="8" t="inlineStr">
-        <is>
-          <t>Caroline S
-(8:00-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="Y5" s="15" t="inlineStr">
-        <is>
-          <t>Mia
-(8:00-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="Z5" s="16" t="inlineStr">
-        <is>
-          <t>Caroline G
-(8:00-12:30 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -928,22 +951,10 @@
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Arya
-(9:00-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="R9" s="8" t="inlineStr">
-        <is>
-          <t>Caroline S
-(9:00-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="T9" s="14" t="inlineStr">
-        <is>
-          <t>Arya
-(9:00-10:30 AM)</t>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Ivanna
+(9:00-12:30 PM)</t>
         </is>
       </c>
     </row>
@@ -953,18 +964,6 @@
           <t>9:15 AM</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Mia
-(9:15-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="J10" s="17" t="inlineStr">
-        <is>
-          <t>Alex
-(9:15-11:00 AM)</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -972,28 +971,46 @@
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Charlotte
 (9:30-12:30 PM)</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Charlie
+(9:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Grace
-(9:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr">
-        <is>
-          <t>Ivanna
-(9:30-11:15 AM)</t>
-        </is>
-      </c>
-      <c r="Q11" s="4" t="inlineStr">
+(9:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Caroline S
+(9:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>Alex
+(9:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>Drew
+(9:30-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
         <is>
           <t>Grace
-(9:30-11:15 AM)</t>
+(9:30-2:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1024,15 +1041,15 @@
           <t>10:30 AM</t>
         </is>
       </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>Drew
-(10:30-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="T15" s="3" t="inlineStr">
-        <is>
-          <t>Charlie
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Keira
+(10:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="L15" s="20" t="inlineStr">
+        <is>
+          <t>Charlotte
 (10:30-12:30 PM)</t>
         </is>
       </c>
@@ -1043,12 +1060,6 @@
           <t>10:45 AM</t>
         </is>
       </c>
-      <c r="L16" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(10:45-2:15 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1056,7 +1067,7 @@
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Caroline G
 (11:00-12:30 PM)</t>
@@ -1064,44 +1075,50 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>Olivia D
+          <t>Caroline G
 (11:00-2:00 PM)</t>
         </is>
       </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>Olivia R
-(11:00-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="J17" s="19" t="inlineStr">
-        <is>
-          <t>Abby
-(11:00-2:15 PM)</t>
-        </is>
-      </c>
-      <c r="K17" s="20" t="inlineStr">
+      <c r="I17" s="20" t="inlineStr">
         <is>
           <t>Charlotte
 (11:00-3:00 PM)</t>
         </is>
       </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>Reese
+(11:00-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="K17" s="19" t="inlineStr">
+        <is>
+          <t>Abby
+(11:00-1:30 PM)</t>
+        </is>
+      </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
           <t>Abby
-(11:00-1:45 PM)</t>
-        </is>
-      </c>
-      <c r="R17" s="20" t="inlineStr">
+(11:00-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>Ivanna
+(11:00-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="S17" s="20" t="inlineStr">
         <is>
           <t>Charlotte
-(11:00-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="U17" s="11" t="inlineStr">
+(11:00-3:00 PM)</t>
+        </is>
+      </c>
+      <c r="U17" s="18" t="inlineStr">
         <is>
           <t>Olivia D
-(11:00-1:15 PM)</t>
+(11:00-3:30 PM)</t>
         </is>
       </c>
     </row>
@@ -1111,24 +1128,6 @@
           <t>11:15 AM</t>
         </is>
       </c>
-      <c r="P18" s="18" t="inlineStr">
-        <is>
-          <t>Reese
-(11:15-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="Q18" s="18" t="inlineStr">
-        <is>
-          <t>Reese
-(11:15-1:15 PM)</t>
-        </is>
-      </c>
-      <c r="S18" s="4" t="inlineStr">
-        <is>
-          <t>Grace
-(11:15-1:15 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1150,7 +1149,7 @@
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Reese
 (12:00-2:00 PM)</t>
@@ -1170,67 +1169,79 @@
           <t>12:30 PM</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Ratna
+(12:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Abby
+(12:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>Caroline S
+(12:30-2:30 PM)</t>
+        </is>
+      </c>
+      <c r="L23" s="14" t="inlineStr">
+        <is>
+          <t>Reese
+(12:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>Laila
-(12:30-2:45 PM)</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
+(12:30-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="inlineStr">
+        <is>
+          <t>Naisha
+(12:30-2:30 PM)</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t>Keira
+(12:30-2:30 PM)</t>
+        </is>
+      </c>
+      <c r="Q23" s="10" t="inlineStr">
+        <is>
+          <t>Arya
+(12:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="R23" s="8" t="inlineStr">
         <is>
           <t>Naisha
 (12:30-3:30 PM)</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Ratna
-(12:30-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Caroline S
-(12:30-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Drew
+      <c r="V23" s="13" t="inlineStr">
+        <is>
+          <t>Keira
 (12:30-5:00 PM)</t>
         </is>
       </c>
-      <c r="N23" s="6" t="inlineStr">
-        <is>
-          <t>Ratna
-(12:30-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="T23" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(12:30-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="V23" s="18" t="inlineStr">
+      <c r="W23" s="14" t="inlineStr">
         <is>
           <t>Reese
 (12:30-5:00 PM)</t>
         </is>
       </c>
-      <c r="X23" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(12:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="Y23" s="12" t="inlineStr">
+      <c r="Y23" s="8" t="inlineStr">
         <is>
           <t>Naisha
 (12:30-5:00 PM)</t>
         </is>
       </c>
-      <c r="Z23" s="17" t="inlineStr">
+      <c r="Z23" s="15" t="inlineStr">
         <is>
           <t>Alex
 (12:30-5:00 PM)</t>
@@ -1250,12 +1261,6 @@
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="O25" s="12" t="inlineStr">
-        <is>
-          <t>Naisha
-(1:00-3:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1263,24 +1268,6 @@
           <t>1:15 PM</t>
         </is>
       </c>
-      <c r="Q26" s="11" t="inlineStr">
-        <is>
-          <t>Olivia D
-(1:15-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="S26" s="12" t="inlineStr">
-        <is>
-          <t>Naisha
-(1:15-2:45 PM)</t>
-        </is>
-      </c>
-      <c r="U26" s="14" t="inlineStr">
-        <is>
-          <t>Arya
-(1:15-3:30 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1288,6 +1275,12 @@
           <t>1:30 PM</t>
         </is>
       </c>
+      <c r="K27" s="10" t="inlineStr">
+        <is>
+          <t>Arya
+(1:30-3:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1295,12 +1288,6 @@
           <t>1:45 PM</t>
         </is>
       </c>
-      <c r="M28" s="10" t="inlineStr">
-        <is>
-          <t>Laila
-(1:45-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1308,51 +1295,63 @@
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Mia
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Olivia R
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Caroline G
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Drew
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Naisha
+(2:00-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Ratna
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>Ivanna
 (2:00-5:00 PM)</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="L29" s="11" t="inlineStr">
+        <is>
+          <t>Caroline G
+(2:00-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="inlineStr">
         <is>
           <t>Olivia R
 (2:00-5:00 PM)</t>
         </is>
       </c>
-      <c r="F29" s="20" t="inlineStr">
-        <is>
-          <t>Charlotte
-(2:00-3:30 PM)</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>Alex
-(2:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr">
-        <is>
-          <t>Charlotte
-(2:00-3:30 PM)</t>
-        </is>
-      </c>
-      <c r="P29" s="15" t="inlineStr">
-        <is>
-          <t>Mia
-(2:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="R29" s="7" t="inlineStr">
-        <is>
-          <t>Ivanna
-(2:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="T29" s="13" t="inlineStr">
-        <is>
-          <t>Olivia R
+      <c r="T29" s="9" t="inlineStr">
+        <is>
+          <t>Ratna
 (2:00-5:00 PM)</t>
         </is>
       </c>
@@ -1363,18 +1362,6 @@
           <t>2:15 PM</t>
         </is>
       </c>
-      <c r="J30" s="14" t="inlineStr">
-        <is>
-          <t>Arya
-(2:15-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="L30" s="16" t="inlineStr">
-        <is>
-          <t>Caroline G
-(2:15-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1382,6 +1369,24 @@
           <t>2:30 PM</t>
         </is>
       </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>Olivia D
+(2:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="O31" s="12" t="inlineStr">
+        <is>
+          <t>Mia
+(2:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>Drew
+(2:30-5:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1389,18 +1394,6 @@
           <t>2:45 PM</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Olivia D
-(2:45-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="S32" s="19" t="inlineStr">
-        <is>
-          <t>Abby
-(2:45-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1408,18 +1401,24 @@
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="K33" s="13" t="inlineStr">
+      <c r="I33" s="15" t="inlineStr">
+        <is>
+          <t>Alex
+(3:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>Grace
+(3:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="S33" s="6" t="inlineStr">
         <is>
           <t>Olivia R
 (3:00-5:00 PM)</t>
         </is>
       </c>
-      <c r="O33" s="5" t="inlineStr">
-        <is>
-          <t>Drew
-(3:00-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1434,30 +1433,36 @@
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
-        <is>
-          <t>Arya
-(3:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="F35" s="16" t="inlineStr">
-        <is>
-          <t>Caroline G
-(3:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="N35" s="6" t="inlineStr">
-        <is>
-          <t>Ratna
-(3:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="U35" s="8" t="inlineStr">
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>Caroline S
 (3:30-5:00 PM)</t>
         </is>
       </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Laila
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="N35" s="13" t="inlineStr">
+        <is>
+          <t>Keira
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="R35" s="18" t="inlineStr">
+        <is>
+          <t>Olivia D
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="U35" s="19" t="inlineStr">
+        <is>
+          <t>Abby
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1494,106 +1499,883 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B43" s="21" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D43" s="21" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E43" s="21" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="G43" s="21" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H43" s="21" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="I43" s="21" t="inlineStr">
+        <is>
+          <t>Closing</t>
+        </is>
+      </c>
+      <c r="J43" s="21" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="K43" s="21" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Abby</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C44" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G44" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G45" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="inlineStr">
+        <is>
+          <t>Arya</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>8</v>
+      </c>
+      <c r="G46" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>Caroline G</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t>Caroline S</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F48" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G48" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>Charlie</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F49" t="n">
+        <v>9</v>
+      </c>
+      <c r="G49" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G50" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>Drew</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G51" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="30" t="inlineStr">
+        <is>
+          <t>Grace</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E52" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G52" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="31" t="inlineStr">
+        <is>
+          <t>Ivanna</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G53" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>Keira</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D54" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G54" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="33" t="inlineStr">
+        <is>
+          <t>Laila</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D55" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G55" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="34" t="inlineStr">
+        <is>
+          <t>Mia</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F56" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G56" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="35" t="inlineStr">
+        <is>
+          <t>Naisha</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" t="n">
+        <v>3</v>
+      </c>
+      <c r="F57" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G57" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="36" t="inlineStr">
+        <is>
+          <t>Olivia D</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E58" t="n">
+        <v>6</v>
+      </c>
+      <c r="F58" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G58" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="37" t="inlineStr">
+        <is>
+          <t>Olivia R</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="n">
+        <v>3</v>
+      </c>
+      <c r="E59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="38" t="inlineStr">
+        <is>
+          <t>Ratna</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C60" t="n">
+        <v>5</v>
+      </c>
+      <c r="D60" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E60" t="n">
+        <v>3</v>
+      </c>
+      <c r="G60" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="39" t="inlineStr">
+        <is>
+          <t>Reese</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D61" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F61" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G61" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="98">
+  <mergeCells count="95">
     <mergeCell ref="L2:M2"/>
+    <mergeCell ref="K17:K26"/>
     <mergeCell ref="V2:W2"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="K3:K10"/>
-    <mergeCell ref="L3:L15"/>
-    <mergeCell ref="T15:T22"/>
-    <mergeCell ref="C10:C22"/>
-    <mergeCell ref="E23:E28"/>
-    <mergeCell ref="J30:J40"/>
+    <mergeCell ref="M17:M28"/>
     <mergeCell ref="V1:Z1"/>
-    <mergeCell ref="E3:E16"/>
-    <mergeCell ref="J3:J9"/>
-    <mergeCell ref="T9:T14"/>
-    <mergeCell ref="H9:H16"/>
-    <mergeCell ref="P18:P28"/>
+    <mergeCell ref="D17:D22"/>
+    <mergeCell ref="H29:H40"/>
+    <mergeCell ref="J29:J40"/>
+    <mergeCell ref="P3:P22"/>
     <mergeCell ref="Q1:U1"/>
-    <mergeCell ref="N29:N34"/>
+    <mergeCell ref="R17:R22"/>
+    <mergeCell ref="L29:L34"/>
     <mergeCell ref="Y23:Y40"/>
     <mergeCell ref="V5:V22"/>
     <mergeCell ref="V23:V40"/>
+    <mergeCell ref="O31:O40"/>
     <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="X23:X40"/>
-    <mergeCell ref="S26:S31"/>
-    <mergeCell ref="P3:P10"/>
-    <mergeCell ref="T3:T8"/>
+    <mergeCell ref="G35:G40"/>
     <mergeCell ref="M3:M16"/>
+    <mergeCell ref="U17:U34"/>
     <mergeCell ref="U35:U40"/>
+    <mergeCell ref="S33:S40"/>
+    <mergeCell ref="E15:E28"/>
+    <mergeCell ref="X5:X40"/>
     <mergeCell ref="Y5:Y22"/>
-    <mergeCell ref="R9:R16"/>
-    <mergeCell ref="B23:B31"/>
-    <mergeCell ref="L30:L40"/>
-    <mergeCell ref="C23:C34"/>
-    <mergeCell ref="Q11:Q17"/>
-    <mergeCell ref="Q18:Q25"/>
-    <mergeCell ref="S18:S25"/>
+    <mergeCell ref="T3:T10"/>
+    <mergeCell ref="N9:N22"/>
+    <mergeCell ref="G11:G16"/>
+    <mergeCell ref="R3:R16"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="J17:J28"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:D20"/>
-    <mergeCell ref="Q3:Q10"/>
+    <mergeCell ref="O3:O10"/>
     <mergeCell ref="D29:D40"/>
     <mergeCell ref="N2:O2"/>
-    <mergeCell ref="F35:F40"/>
+    <mergeCell ref="F11:F22"/>
     <mergeCell ref="G17:G28"/>
-    <mergeCell ref="P29:P40"/>
-    <mergeCell ref="R29:R40"/>
-    <mergeCell ref="M17:M27"/>
-    <mergeCell ref="H17:H22"/>
+    <mergeCell ref="R23:R34"/>
+    <mergeCell ref="L35:L40"/>
+    <mergeCell ref="T29:T40"/>
     <mergeCell ref="L1:P1"/>
-    <mergeCell ref="T29:T40"/>
-    <mergeCell ref="W5:W40"/>
-    <mergeCell ref="O3:O24"/>
-    <mergeCell ref="G3:G16"/>
-    <mergeCell ref="H3:H8"/>
-    <mergeCell ref="R3:R8"/>
+    <mergeCell ref="C23:C28"/>
+    <mergeCell ref="S17:S32"/>
+    <mergeCell ref="I3:I16"/>
     <mergeCell ref="G1:K1"/>
-    <mergeCell ref="S3:S17"/>
-    <mergeCell ref="F29:F34"/>
-    <mergeCell ref="F3:F22"/>
+    <mergeCell ref="H11:H28"/>
+    <mergeCell ref="D23:D28"/>
+    <mergeCell ref="O23:O30"/>
+    <mergeCell ref="H3:H10"/>
+    <mergeCell ref="J3:J10"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="G29:G40"/>
+    <mergeCell ref="O11:O22"/>
+    <mergeCell ref="D3:D16"/>
     <mergeCell ref="K33:K40"/>
-    <mergeCell ref="I11:I40"/>
     <mergeCell ref="Z23:Z40"/>
-    <mergeCell ref="C35:C40"/>
-    <mergeCell ref="O33:O40"/>
-    <mergeCell ref="D21:D28"/>
+    <mergeCell ref="M29:M40"/>
+    <mergeCell ref="B21:B28"/>
+    <mergeCell ref="K11:K16"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="I3:I10"/>
-    <mergeCell ref="F23:F28"/>
-    <mergeCell ref="B11:B22"/>
-    <mergeCell ref="O25:O32"/>
-    <mergeCell ref="J10:J16"/>
-    <mergeCell ref="U3:U10"/>
-    <mergeCell ref="P11:P17"/>
-    <mergeCell ref="K17:K32"/>
-    <mergeCell ref="B3:B10"/>
-    <mergeCell ref="X5:X22"/>
+    <mergeCell ref="W23:W40"/>
+    <mergeCell ref="P31:P40"/>
+    <mergeCell ref="R35:R40"/>
+    <mergeCell ref="L15:L22"/>
+    <mergeCell ref="G3:G10"/>
+    <mergeCell ref="C3:C22"/>
+    <mergeCell ref="F23:F30"/>
+    <mergeCell ref="U3:U12"/>
+    <mergeCell ref="G29:G34"/>
+    <mergeCell ref="Q3:Q22"/>
+    <mergeCell ref="B3:B20"/>
+    <mergeCell ref="N23:N34"/>
+    <mergeCell ref="I17:I32"/>
+    <mergeCell ref="E3:E14"/>
+    <mergeCell ref="T11:T28"/>
     <mergeCell ref="N35:N40"/>
     <mergeCell ref="Z5:Z22"/>
     <mergeCell ref="S2:T2"/>
-    <mergeCell ref="E17:E22"/>
-    <mergeCell ref="Q26:Q40"/>
-    <mergeCell ref="M28:M40"/>
-    <mergeCell ref="S32:S40"/>
-    <mergeCell ref="H23:H40"/>
-    <mergeCell ref="N23:N28"/>
-    <mergeCell ref="U26:U34"/>
-    <mergeCell ref="C3:C9"/>
-    <mergeCell ref="N3:N14"/>
+    <mergeCell ref="N3:N8"/>
+    <mergeCell ref="S3:S16"/>
+    <mergeCell ref="J11:J16"/>
+    <mergeCell ref="L23:L28"/>
+    <mergeCell ref="F3:F10"/>
+    <mergeCell ref="K27:K32"/>
+    <mergeCell ref="L3:L14"/>
+    <mergeCell ref="C29:C40"/>
     <mergeCell ref="E29:E40"/>
-    <mergeCell ref="L16:L29"/>
-    <mergeCell ref="B32:B40"/>
-    <mergeCell ref="T23:T28"/>
-    <mergeCell ref="J17:J29"/>
-    <mergeCell ref="U17:U25"/>
-    <mergeCell ref="N15:N22"/>
-    <mergeCell ref="R17:R28"/>
+    <mergeCell ref="I33:I40"/>
+    <mergeCell ref="B29:B40"/>
+    <mergeCell ref="P23:P30"/>
+    <mergeCell ref="W5:W22"/>
+    <mergeCell ref="F31:F40"/>
+    <mergeCell ref="Q23:Q40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
implemented max shift limit
</commit_message>
<xml_diff>
--- a/data/generated_schedule.xlsx
+++ b/data/generated_schedule.xlsx
@@ -63,6 +63,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D6B656"/>
+        <bgColor rgb="00D6B656"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00674EA7"/>
+        <bgColor rgb="00674EA7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A64D79"/>
+        <bgColor rgb="00A64D79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF9000"/>
+        <bgColor rgb="00BF9000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6699"/>
+        <bgColor rgb="00FF6699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+        <bgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00548235"/>
         <bgColor rgb="00548235"/>
       </patternFill>
@@ -75,32 +111,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BF9000"/>
-        <bgColor rgb="00BF9000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="007030A0"/>
         <bgColor rgb="007030A0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00674EA7"/>
-        <bgColor rgb="00674EA7"/>
+        <fgColor rgb="00ED7D31"/>
+        <bgColor rgb="00ED7D31"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6B656"/>
-        <bgColor rgb="00D6B656"/>
+        <fgColor rgb="009E480E"/>
+        <bgColor rgb="009E480E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0070AD47"/>
-        <bgColor rgb="0070AD47"/>
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+        <bgColor rgb="00375623"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,50 +153,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A64D79"/>
-        <bgColor rgb="00A64D79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
-        <bgColor rgb="00C00000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF6699"/>
-        <bgColor rgb="00FF6699"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ED7D31"/>
-        <bgColor rgb="00ED7D31"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
         <bgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="009E480E"/>
-        <bgColor rgb="009E480E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00375623"/>
-        <bgColor rgb="00375623"/>
       </patternFill>
     </fill>
   </fills>
@@ -178,16 +178,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,31 +196,19 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -229,28 +217,40 @@
     <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -761,26 +761,26 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Drew
-(7:30-9:45 AM)</t>
+          <t>Ratna
+(7:30-10:30 AM)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Reese
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Grace
 (7:30-12:30 PM)</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Mia
-(7:30-11:00 AM)</t>
-        </is>
-      </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Ratna
-(7:30-11:00 AM)</t>
+          <t>Olivia R
+(7:30-10:00 AM)</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -791,92 +791,92 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
+          <t>Arya
+(7:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Naisha
+(7:30-9:00 AM)</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
           <t>Alex
-(7:30-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
+(7:30-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>Keira
-(7:30-9:15 AM)</t>
-        </is>
-      </c>
-      <c r="I3" s="10" t="inlineStr">
+(7:30-9:30 AM)</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
         <is>
           <t>Caroline G
 (7:30-9:30 AM)</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Drew
+(7:30-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="M3" s="14" t="inlineStr">
+        <is>
+          <t>Mia
+(7:30-12:15 PM)</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>Ivanna
+(7:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Ratna
+(7:30-9:45 AM)</t>
+        </is>
+      </c>
+      <c r="P3" s="15" t="inlineStr">
+        <is>
+          <t>Laila
+(7:30-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="Q3" s="15" t="inlineStr">
+        <is>
+          <t>Laila
 (7:30-9:30 AM)</t>
         </is>
       </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>Abby
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="L3" s="12" t="inlineStr">
-        <is>
-          <t>Laila
-(7:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>Mia
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>Drew
-(7:30-12:15 PM)</t>
-        </is>
-      </c>
-      <c r="O3" s="13" t="inlineStr">
-        <is>
-          <t>Reese
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Ratna
 (7:30-9:15 AM)</t>
         </is>
       </c>
-      <c r="P3" s="14" t="inlineStr">
-        <is>
-          <t>Olivia R
-(7:30-10:15 AM)</t>
-        </is>
-      </c>
-      <c r="Q3" s="15" t="inlineStr">
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Arya
+(7:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="T3" s="16" t="inlineStr">
         <is>
           <t>Caroline S
 (7:30-11:00 AM)</t>
         </is>
       </c>
-      <c r="R3" s="12" t="inlineStr">
-        <is>
-          <t>Laila
+      <c r="U3" s="17" t="inlineStr">
+        <is>
+          <t>Olivia D
 (7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="S3" s="16" t="inlineStr">
-        <is>
-          <t>Arya
-(7:30-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="T3" s="17" t="inlineStr">
-        <is>
-          <t>Naisha
-(7:30-9:30 AM)</t>
-        </is>
-      </c>
-      <c r="U3" s="11" t="inlineStr">
-        <is>
-          <t>Abby
-(7:30-9:15 AM)</t>
         </is>
       </c>
     </row>
@@ -893,36 +893,36 @@
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="V5" s="5" t="inlineStr">
+      <c r="V5" s="14" t="inlineStr">
         <is>
           <t>Mia
 (8:00-12:30 PM)</t>
         </is>
       </c>
-      <c r="W5" s="18" t="inlineStr">
+      <c r="W5" s="17" t="inlineStr">
         <is>
           <t>Olivia D
 (8:00-12:30 PM)</t>
         </is>
       </c>
-      <c r="X5" s="15" t="inlineStr">
+      <c r="X5" s="18" t="inlineStr">
+        <is>
+          <t>Abby
+(8:00-12:30 PM)</t>
+        </is>
+      </c>
+      <c r="Y5" s="19" t="inlineStr">
+        <is>
+          <t>Charlie
+(8:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="Z5" s="16" t="inlineStr">
         <is>
           <t>Caroline S
 (8:00-12:30 PM)</t>
         </is>
       </c>
-      <c r="Y5" s="19" t="inlineStr">
-        <is>
-          <t>Charlie
-(8:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="Z5" s="11" t="inlineStr">
-        <is>
-          <t>Abby
-(8:00-12:30 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -951,6 +951,12 @@
           <t>9:00 AM</t>
         </is>
       </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>Caroline S
+(9:00-11:00 AM)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -958,22 +964,10 @@
           <t>9:15 AM</t>
         </is>
       </c>
-      <c r="H10" s="16" t="inlineStr">
-        <is>
-          <t>Arya
-(9:15-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="O10" s="16" t="inlineStr">
-        <is>
-          <t>Arya
-(9:15-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="U10" s="19" t="inlineStr">
+      <c r="R10" s="19" t="inlineStr">
         <is>
           <t>Charlie
-(9:15-11:15 AM)</t>
+(9:15-11:30 AM)</t>
         </is>
       </c>
     </row>
@@ -983,36 +977,30 @@
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="I11" s="15" t="inlineStr">
-        <is>
-          <t>Caroline S
-(9:30-11:00 AM)</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Grace
-(9:30-11:15 AM)</t>
-        </is>
-      </c>
-      <c r="M11" s="20" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Charlotte
 (9:30-12:30 PM)</t>
         </is>
       </c>
-      <c r="R11" s="4" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Grace
+(9:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="Q11" s="10" t="inlineStr">
+        <is>
+          <t>Alex
+(9:30-11:00 AM)</t>
+        </is>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
         <is>
           <t>Grace
 (9:30-12:15 PM)</t>
         </is>
       </c>
-      <c r="T11" s="8" t="inlineStr">
-        <is>
-          <t>Alex
-(9:30-11:30 AM)</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1020,10 +1008,10 @@
           <t>9:45 AM</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="O12" s="20" t="inlineStr">
         <is>
           <t>Charlotte
-(9:45-12:30 PM)</t>
+(9:45-12:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1033,6 +1021,12 @@
           <t>10:00 AM</t>
         </is>
       </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Drew
+(10:00-11:30 AM)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1040,12 +1034,6 @@
           <t>10:15 AM</t>
         </is>
       </c>
-      <c r="P14" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(10:15-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1053,6 +1041,12 @@
           <t>10:30 AM</t>
         </is>
       </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Keira
+(10:30-2:15 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1067,58 +1061,52 @@
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Caroline G
-(11:00-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>Reese
-(11:00-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>Caroline G
-(11:00-1:15 PM)</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>Reese
-(11:00-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="I17" s="18" t="inlineStr">
-        <is>
-          <t>Olivia D
-(11:00-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="K17" s="14" t="inlineStr">
-        <is>
-          <t>Olivia R
-(11:00-12:30 PM)</t>
-        </is>
-      </c>
-      <c r="O17" s="11" t="inlineStr">
+      <c r="G17" s="18" t="inlineStr">
         <is>
           <t>Abby
 (11:00-2:00 PM)</t>
         </is>
       </c>
-      <c r="Q17" s="20" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Reese
+(11:00-1:15 PM)</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Caroline G
+(11:00-1:00 PM)</t>
+        </is>
+      </c>
+      <c r="K17" s="20" t="inlineStr">
         <is>
           <t>Charlotte
 (11:00-3:00 PM)</t>
         </is>
       </c>
+      <c r="N17" s="18" t="inlineStr">
+        <is>
+          <t>Abby
+(11:00-1:15 PM)</t>
+        </is>
+      </c>
+      <c r="Q17" s="20" t="inlineStr">
+        <is>
+          <t>Charlotte
+(11:00-2:45 PM)</t>
+        </is>
+      </c>
       <c r="S17" s="12" t="inlineStr">
         <is>
-          <t>Laila
-(11:00-12:30 PM)</t>
+          <t>Caroline G
+(11:00-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="T17" s="17" t="inlineStr">
+        <is>
+          <t>Olivia D
+(11:00-2:30 PM)</t>
         </is>
       </c>
     </row>
@@ -1128,18 +1116,6 @@
           <t>11:15 AM</t>
         </is>
       </c>
-      <c r="J18" s="20" t="inlineStr">
-        <is>
-          <t>Charlotte
-(11:15-2:15 PM)</t>
-        </is>
-      </c>
-      <c r="U18" s="13" t="inlineStr">
-        <is>
-          <t>Reese
-(11:15-1:30 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1147,10 +1123,16 @@
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="T19" s="18" t="inlineStr">
-        <is>
-          <t>Olivia D
-(11:30-5:00 PM)</t>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Reese
+(11:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="R19" s="11" t="inlineStr">
+        <is>
+          <t>Keira
+(11:30-2:00 PM)</t>
         </is>
       </c>
     </row>
@@ -1167,6 +1149,12 @@
           <t>12:00 PM</t>
         </is>
       </c>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>Alex
+(12:00-2:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1174,15 +1162,15 @@
           <t>12:15 PM</t>
         </is>
       </c>
-      <c r="N22" s="17" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Reese
+(12:15-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="U22" s="9" t="inlineStr">
         <is>
           <t>Naisha
-(12:15-2:15 PM)</t>
-        </is>
-      </c>
-      <c r="R22" s="10" t="inlineStr">
-        <is>
-          <t>Caroline G
 (12:15-2:00 PM)</t>
         </is>
       </c>
@@ -1193,78 +1181,60 @@
           <t>12:30 PM</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Caroline S
-(12:30-2:15 PM)</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Ratna
 (12:30-2:00 PM)</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Alex
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Caroline S
 (12:30-2:00 PM)</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Naisha
+(12:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Drew
+(12:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Naisha
+(12:30-2:00 PM)</t>
+        </is>
+      </c>
+      <c r="V23" s="11" t="inlineStr">
+        <is>
+          <t>Keira
+(12:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="W23" s="9" t="inlineStr">
         <is>
           <t>Naisha
 (12:30-5:00 PM)</t>
         </is>
       </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>Arya
-(12:30-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>Drew
-(12:30-3:30 PM)</t>
-        </is>
-      </c>
-      <c r="M23" s="8" t="inlineStr">
+      <c r="X23" s="10" t="inlineStr">
         <is>
           <t>Alex
-(12:30-2:00 PM)</t>
-        </is>
-      </c>
-      <c r="S23" s="16" t="inlineStr">
-        <is>
-          <t>Arya
 (12:30-5:00 PM)</t>
         </is>
       </c>
-      <c r="V23" s="17" t="inlineStr">
-        <is>
-          <t>Naisha
-(12:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="W23" s="13" t="inlineStr">
+      <c r="Z23" s="4" t="inlineStr">
         <is>
           <t>Reese
 (12:30-5:00 PM)</t>
         </is>
       </c>
-      <c r="X23" s="9" t="inlineStr">
-        <is>
-          <t>Keira
-(12:30-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="Z23" s="8" t="inlineStr">
-        <is>
-          <t>Alex
-(12:30-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1279,6 +1249,12 @@
           <t>1:00 PM</t>
         </is>
       </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>Naisha
+(1:00-3:15 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1286,10 +1262,16 @@
           <t>1:15 PM</t>
         </is>
       </c>
-      <c r="G26" s="19" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Grace
+(1:15-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="N26" s="19" t="inlineStr">
         <is>
           <t>Charlie
-(1:15-3:15 PM)</t>
+(1:15-2:45 PM)</t>
         </is>
       </c>
     </row>
@@ -1299,12 +1281,6 @@
           <t>1:30 PM</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr">
-        <is>
-          <t>Grace
-(1:30-5:00 PM)</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1319,52 +1295,76 @@
           <t>2:00 PM</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Caroline G
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Arya
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Olivia D
+(2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Olivia R
 (2:00-5:00 PM)</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Drew
-(2:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Ivanna
 (2:00-5:00 PM)</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>Ratna
-(2:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="I29" s="7" t="inlineStr">
-        <is>
-          <t>Ivanna
-(2:00-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="M29" s="14" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Olivia R
 (2:00-5:00 PM)</t>
         </is>
       </c>
-      <c r="O29" s="5" t="inlineStr">
-        <is>
-          <t>Mia
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>Caroline G
+(2:00-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>Olivia R
+(2:00-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="O29" s="8" t="inlineStr">
+        <is>
+          <t>Arya
 (2:00-5:00 PM)</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
         <is>
-          <t>Ratna
+          <t>Olivia R
 (2:00-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="S29" s="15" t="inlineStr">
+        <is>
+          <t>Laila
+(2:00-3:30 PM)</t>
+        </is>
+      </c>
+      <c r="U29" s="7" t="inlineStr">
+        <is>
+          <t>Ivanna
+(2:00-3:30 PM)</t>
         </is>
       </c>
     </row>
@@ -1374,21 +1374,9 @@
           <t>2:15 PM</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Caroline G
-(2:15-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="J30" s="14" t="inlineStr">
-        <is>
-          <t>Olivia R
-(2:15-5:00 PM)</t>
-        </is>
-      </c>
-      <c r="N30" s="10" t="inlineStr">
-        <is>
-          <t>Caroline G
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Drew
 (2:15-5:00 PM)</t>
         </is>
       </c>
@@ -1399,6 +1387,12 @@
           <t>2:30 PM</t>
         </is>
       </c>
+      <c r="T31" s="3" t="inlineStr">
+        <is>
+          <t>Ratna
+(2:30-5:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1406,6 +1400,18 @@
           <t>2:45 PM</t>
         </is>
       </c>
+      <c r="N32" s="14" t="inlineStr">
+        <is>
+          <t>Mia
+(2:45-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="Q32" s="13" t="inlineStr">
+        <is>
+          <t>Drew
+(2:45-5:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1413,9 +1419,9 @@
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="Q33" s="7" t="inlineStr">
-        <is>
-          <t>Ivanna
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Ratna
 (3:00-5:00 PM)</t>
         </is>
       </c>
@@ -1426,7 +1432,7 @@
           <t>3:15 PM</t>
         </is>
       </c>
-      <c r="G34" s="11" t="inlineStr">
+      <c r="J34" s="18" t="inlineStr">
         <is>
           <t>Abby
 (3:15-5:00 PM)</t>
@@ -1439,12 +1445,36 @@
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="K35" s="15" t="inlineStr">
+      <c r="L35" s="18" t="inlineStr">
+        <is>
+          <t>Abby
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="M35" s="15" t="inlineStr">
+        <is>
+          <t>Laila
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="P35" s="12" t="inlineStr">
+        <is>
+          <t>Caroline G
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
+      <c r="S35" s="16" t="inlineStr">
         <is>
           <t>Caroline S
 (3:30-5:00 PM)</t>
         </is>
       </c>
+      <c r="U35" s="14" t="inlineStr">
+        <is>
+          <t>Mia
+(3:30-5:00 PM)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1545,13 +1575,10 @@
         </is>
       </c>
       <c r="C44" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="D44" t="n">
         <v>3.75</v>
-      </c>
-      <c r="D44" t="n">
-        <v>3</v>
-      </c>
-      <c r="E44" t="n">
-        <v>1.75</v>
       </c>
       <c r="F44" t="n">
         <v>4.5</v>
@@ -1586,17 +1613,14 @@
           <t>Alex</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" t="n">
         <v>1.5</v>
-      </c>
-      <c r="C45" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="D45" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E45" t="n">
-        <v>2</v>
       </c>
       <c r="F45" t="n">
         <v>4.5</v>
@@ -1631,14 +1655,17 @@
           <t>Arya</t>
         </is>
       </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
       <c r="C46" t="n">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="D46" t="n">
-        <v>1.75</v>
+        <v>3</v>
       </c>
       <c r="E46" t="n">
-        <v>8</v>
+        <v>3.5</v>
       </c>
       <c r="G46" s="21" t="n">
         <v>13</v>
@@ -1671,16 +1698,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4.25</v>
+        <v>3</v>
       </c>
       <c r="C47" t="n">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
-        <v>1.75</v>
+        <v>3</v>
       </c>
       <c r="G47" s="21" t="n">
         <v>13</v>
@@ -1713,19 +1740,19 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.75</v>
+        <v>1.5</v>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>4.5</v>
       </c>
       <c r="G48" s="21" t="n">
-        <v>12.75</v>
+        <v>13</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -1754,17 +1781,17 @@
           <t>Charlie</t>
         </is>
       </c>
-      <c r="C49" t="n">
-        <v>2</v>
+      <c r="D49" t="n">
+        <v>1.5</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="F49" t="n">
         <v>9</v>
       </c>
       <c r="G49" s="21" t="n">
-        <v>13</v>
+        <v>12.75</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -1794,19 +1821,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>2.25</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="G50" s="21" t="n">
-        <v>12.75</v>
+        <v>13</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -1836,13 +1863,16 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5.25</v>
+        <v>4.25</v>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="D51" t="n">
-        <v>4.75</v>
+        <v>5</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2.25</v>
       </c>
       <c r="G51" s="21" t="n">
         <v>13</v>
@@ -1878,10 +1908,10 @@
         <v>5</v>
       </c>
       <c r="C52" t="n">
-        <v>1.75</v>
+        <v>5.25</v>
       </c>
       <c r="E52" t="n">
-        <v>6.25</v>
+        <v>2.75</v>
       </c>
       <c r="G52" s="21" t="n">
         <v>13</v>
@@ -1914,13 +1944,16 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C53" t="n">
         <v>3</v>
       </c>
+      <c r="D53" t="n">
+        <v>3.5</v>
+      </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G53" s="21" t="n">
         <v>13</v>
@@ -1952,17 +1985,20 @@
           <t>Keira</t>
         </is>
       </c>
+      <c r="B54" t="n">
+        <v>3.75</v>
+      </c>
       <c r="C54" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="D54" t="n">
-        <v>6.75</v>
+        <v>2</v>
+      </c>
+      <c r="E54" t="n">
+        <v>2.5</v>
       </c>
       <c r="F54" t="n">
         <v>4.5</v>
       </c>
       <c r="G54" s="21" t="n">
-        <v>13</v>
+        <v>12.75</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2027,11 +2063,11 @@
           <t>Mia</t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>3.5</v>
-      </c>
       <c r="D56" t="n">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1.5</v>
       </c>
       <c r="F56" t="n">
         <v>4.5</v>
@@ -2067,13 +2103,16 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>4.5</v>
+        <v>1.5</v>
+      </c>
+      <c r="C57" t="n">
+        <v>3.75</v>
       </c>
       <c r="D57" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="F57" t="n">
         <v>4.5</v>
@@ -2108,7 +2147,7 @@
           <t>Olivia D</t>
         </is>
       </c>
-      <c r="C58" t="n">
+      <c r="B58" t="n">
         <v>3</v>
       </c>
       <c r="E58" t="n">
@@ -2148,13 +2187,16 @@
         </is>
       </c>
       <c r="B59" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C59" t="n">
         <v>3</v>
       </c>
-      <c r="C59" t="n">
-        <v>4.25</v>
-      </c>
       <c r="D59" t="n">
-        <v>5.75</v>
+        <v>1.5</v>
+      </c>
+      <c r="E59" t="n">
+        <v>3</v>
       </c>
       <c r="G59" s="21" t="n">
         <v>13</v>
@@ -2187,13 +2229,16 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="C60" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="D60" t="n">
+        <v>2.25</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>4.25</v>
       </c>
       <c r="G60" s="21" t="n">
         <v>13</v>
@@ -2226,17 +2271,14 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="C61" t="n">
-        <v>1.5</v>
+        <v>2.25</v>
       </c>
       <c r="D61" t="n">
         <v>1.75</v>
       </c>
-      <c r="E61" t="n">
-        <v>2.25</v>
-      </c>
       <c r="F61" t="n">
         <v>4.5</v>
       </c>
@@ -2265,99 +2307,104 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="92">
+  <mergeCells count="97">
     <mergeCell ref="L2:M2"/>
-    <mergeCell ref="S23:S40"/>
+    <mergeCell ref="S35:S40"/>
     <mergeCell ref="V2:W2"/>
+    <mergeCell ref="N26:N31"/>
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="K3:K10"/>
-    <mergeCell ref="J30:J40"/>
-    <mergeCell ref="O17:O28"/>
+    <mergeCell ref="C3:C10"/>
+    <mergeCell ref="I3:I22"/>
+    <mergeCell ref="P35:P40"/>
+    <mergeCell ref="E13:E18"/>
     <mergeCell ref="V1:Z1"/>
-    <mergeCell ref="D17:D22"/>
-    <mergeCell ref="H3:H9"/>
-    <mergeCell ref="N3:N21"/>
-    <mergeCell ref="E3:E16"/>
-    <mergeCell ref="H29:H40"/>
-    <mergeCell ref="E17:E28"/>
+    <mergeCell ref="O12:O20"/>
+    <mergeCell ref="R3:R9"/>
+    <mergeCell ref="H9:H16"/>
     <mergeCell ref="Q1:U1"/>
+    <mergeCell ref="L29:L34"/>
+    <mergeCell ref="B15:B29"/>
     <mergeCell ref="V5:V22"/>
     <mergeCell ref="V23:V40"/>
-    <mergeCell ref="K17:K22"/>
     <mergeCell ref="Q2:R2"/>
     <mergeCell ref="X23:X40"/>
     <mergeCell ref="O29:O40"/>
-    <mergeCell ref="G26:G33"/>
-    <mergeCell ref="G34:G40"/>
-    <mergeCell ref="H23:H28"/>
-    <mergeCell ref="F23:F40"/>
-    <mergeCell ref="T3:T10"/>
-    <mergeCell ref="B23:B29"/>
-    <mergeCell ref="U3:U9"/>
-    <mergeCell ref="I11:I16"/>
+    <mergeCell ref="Q17:Q31"/>
+    <mergeCell ref="J34:J40"/>
+    <mergeCell ref="U35:U40"/>
+    <mergeCell ref="M22:M28"/>
+    <mergeCell ref="T31:T40"/>
+    <mergeCell ref="H26:H40"/>
+    <mergeCell ref="T17:T30"/>
+    <mergeCell ref="E3:E12"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="T3:T16"/>
+    <mergeCell ref="Q3:Q10"/>
     <mergeCell ref="D29:D40"/>
     <mergeCell ref="N2:O2"/>
+    <mergeCell ref="G17:G28"/>
     <mergeCell ref="R29:R40"/>
-    <mergeCell ref="P14:P40"/>
-    <mergeCell ref="U27:U40"/>
-    <mergeCell ref="H17:H22"/>
+    <mergeCell ref="L35:L40"/>
     <mergeCell ref="L1:P1"/>
+    <mergeCell ref="O3:O11"/>
     <mergeCell ref="C23:C28"/>
-    <mergeCell ref="M23:M28"/>
+    <mergeCell ref="R10:R18"/>
     <mergeCell ref="G3:G16"/>
+    <mergeCell ref="H3:H8"/>
+    <mergeCell ref="O21:O28"/>
     <mergeCell ref="G1:K1"/>
-    <mergeCell ref="B3:B11"/>
-    <mergeCell ref="J11:J17"/>
     <mergeCell ref="D23:D28"/>
     <mergeCell ref="J3:J10"/>
     <mergeCell ref="F3:F22"/>
     <mergeCell ref="G2:H2"/>
+    <mergeCell ref="J17:J24"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="D3:D16"/>
+    <mergeCell ref="H17:H25"/>
+    <mergeCell ref="G29:G40"/>
     <mergeCell ref="I29:I40"/>
-    <mergeCell ref="K23:K34"/>
-    <mergeCell ref="U10:U17"/>
+    <mergeCell ref="K33:K40"/>
     <mergeCell ref="Z23:Z40"/>
-    <mergeCell ref="J18:J29"/>
-    <mergeCell ref="U18:U26"/>
-    <mergeCell ref="N22:N29"/>
-    <mergeCell ref="M29:M40"/>
-    <mergeCell ref="S17:S22"/>
-    <mergeCell ref="Q33:Q40"/>
+    <mergeCell ref="F29:F40"/>
+    <mergeCell ref="J25:J33"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="I3:I10"/>
+    <mergeCell ref="F23:F28"/>
     <mergeCell ref="W23:W40"/>
-    <mergeCell ref="O3:O9"/>
+    <mergeCell ref="U22:U28"/>
+    <mergeCell ref="S17:S28"/>
     <mergeCell ref="Y5:Y40"/>
-    <mergeCell ref="C3:C22"/>
-    <mergeCell ref="H10:H16"/>
-    <mergeCell ref="N30:N40"/>
-    <mergeCell ref="M3:M10"/>
-    <mergeCell ref="R3:R10"/>
+    <mergeCell ref="M3:M21"/>
+    <mergeCell ref="N3:N16"/>
+    <mergeCell ref="E19:E28"/>
+    <mergeCell ref="N32:N40"/>
+    <mergeCell ref="I23:I28"/>
+    <mergeCell ref="U3:U10"/>
+    <mergeCell ref="M29:M34"/>
+    <mergeCell ref="U11:U21"/>
+    <mergeCell ref="P3:P34"/>
+    <mergeCell ref="L3:L22"/>
+    <mergeCell ref="C11:C22"/>
+    <mergeCell ref="N17:N25"/>
+    <mergeCell ref="K17:K32"/>
     <mergeCell ref="X5:X22"/>
     <mergeCell ref="Z5:Z22"/>
     <mergeCell ref="S2:T2"/>
-    <mergeCell ref="K35:K40"/>
-    <mergeCell ref="Q17:Q32"/>
-    <mergeCell ref="Q3:Q16"/>
+    <mergeCell ref="D3:D22"/>
+    <mergeCell ref="M35:M40"/>
     <mergeCell ref="S3:S16"/>
-    <mergeCell ref="R22:R28"/>
-    <mergeCell ref="O10:O16"/>
+    <mergeCell ref="B3:B14"/>
+    <mergeCell ref="J11:J16"/>
+    <mergeCell ref="R19:R28"/>
+    <mergeCell ref="L23:L28"/>
     <mergeCell ref="B30:B40"/>
-    <mergeCell ref="P3:P13"/>
     <mergeCell ref="C29:C40"/>
-    <mergeCell ref="M11:M22"/>
     <mergeCell ref="E29:E40"/>
-    <mergeCell ref="T19:T40"/>
-    <mergeCell ref="L3:L40"/>
-    <mergeCell ref="T11:T18"/>
+    <mergeCell ref="Q32:Q40"/>
     <mergeCell ref="W5:W22"/>
-    <mergeCell ref="G17:G25"/>
-    <mergeCell ref="I17:I28"/>
-    <mergeCell ref="B12:B22"/>
-    <mergeCell ref="R11:R21"/>
+    <mergeCell ref="Q11:Q16"/>
+    <mergeCell ref="S29:S34"/>
+    <mergeCell ref="U29:U34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>